<commit_message>
Adicionar resoluções e alternativas do Projeto Final
</commit_message>
<xml_diff>
--- a/assets/ficheiros/Excel/UFCD0778_Livro2_Formatacao_Apresentacao.xlsx
+++ b/assets/ficheiros/Excel/UFCD0778_Livro2_Formatacao_Apresentacao.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7157BA52-D70E-4876-A960-B10B0BA566B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="465" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="465" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INSTRUÇÕES" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="DESAFIO" sheetId="6" r:id="rId6"/>
     <sheet name="VERIFICAÇÃO" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
@@ -1264,7 +1264,20 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1278,19 +1291,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1540,44 +1540,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="1"/>
@@ -1592,114 +1592,114 @@
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" ht="15.75">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="34"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
     </row>
     <row r="6" spans="1:10" ht="30.95" customHeight="1">
       <c r="A6" s="2">
         <v>1</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="35"/>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="35"/>
-      <c r="J6" s="35"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
     </row>
     <row r="7" spans="1:10" ht="30.95" customHeight="1">
       <c r="A7" s="2">
         <v>2</v>
       </c>
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
     </row>
     <row r="8" spans="1:10" ht="30.95" customHeight="1">
       <c r="A8" s="2">
         <v>3</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="35"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:10" ht="30.95" customHeight="1">
       <c r="A9" s="2">
         <v>4</v>
       </c>
-      <c r="B9" s="35" t="s">
+      <c r="B9" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="35"/>
-      <c r="I9" s="35"/>
-      <c r="J9" s="35"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
     </row>
     <row r="10" spans="1:10" ht="30.95" customHeight="1">
       <c r="A10" s="2">
         <v>5</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="B10" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-      <c r="J10" s="35"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
     </row>
     <row r="11" spans="1:10" ht="30.95" customHeight="1">
       <c r="A11" s="2">
         <v>6</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="35"/>
-      <c r="J11" s="35"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="1"/>
@@ -1726,56 +1726,56 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" ht="15.75">
-      <c r="A14" s="36" t="s">
+      <c r="A14" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="34"/>
-      <c r="B17" s="34"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="34"/>
-      <c r="I17" s="34"/>
-      <c r="J17" s="34"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="1"/>
@@ -3975,17 +3975,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A5:J5"/>
-    <mergeCell ref="B6:J6"/>
-    <mergeCell ref="B7:J7"/>
     <mergeCell ref="A15:J17"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="A14:J14"/>
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A5:J5"/>
+    <mergeCell ref="B6:J6"/>
+    <mergeCell ref="B7:J7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4010,64 +4010,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
     </row>
     <row r="2" spans="1:12">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="34"/>
-      <c r="L2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
     </row>
     <row r="4" spans="1:12">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="1"/>
@@ -7479,56 +7479,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" customHeight="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="36" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
     </row>
     <row r="2" spans="1:10" ht="21" customHeight="1">
-      <c r="A2" s="30"/>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="A2" s="35"/>
+      <c r="B2" s="35"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
     </row>
     <row r="3" spans="1:10" ht="21" customHeight="1">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
     </row>
     <row r="4" spans="1:10" ht="21" customHeight="1">
-      <c r="A4" s="30"/>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="30"/>
-      <c r="F4" s="30"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
     </row>
     <row r="5" spans="1:10" ht="21" customHeight="1">
       <c r="A5" s="16"/>
@@ -7543,31 +7543,31 @@
       <c r="J5" s="16"/>
     </row>
     <row r="6" spans="1:10" ht="21" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="37"/>
       <c r="J6" s="16"/>
     </row>
     <row r="7" spans="1:10" ht="21" customHeight="1">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="37"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="37"/>
       <c r="J7" s="16"/>
     </row>
     <row r="8" spans="1:10" ht="21" customHeight="1">
@@ -8447,17 +8447,17 @@
       </c>
     </row>
     <row r="36" spans="1:10" ht="21" customHeight="1">
-      <c r="A36" s="33" t="s">
+      <c r="A36" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="B36" s="33"/>
-      <c r="C36" s="33"/>
-      <c r="D36" s="33"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="33"/>
-      <c r="G36" s="33"/>
-      <c r="H36" s="33"/>
-      <c r="I36" s="33"/>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
       <c r="J36" s="16"/>
     </row>
     <row r="37" spans="1:10" ht="21" customHeight="1">
@@ -8799,29 +8799,29 @@
       <c r="J51" s="16"/>
     </row>
     <row r="52" spans="1:10" ht="30" customHeight="1">
-      <c r="A52" s="29" t="s">
+      <c r="A52" s="31" t="s">
         <v>170</v>
       </c>
-      <c r="B52" s="30"/>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="30"/>
-      <c r="F52" s="30"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30"/>
-      <c r="I52" s="30"/>
+      <c r="B52" s="35"/>
+      <c r="C52" s="35"/>
+      <c r="D52" s="35"/>
+      <c r="E52" s="35"/>
+      <c r="F52" s="35"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="35"/>
+      <c r="I52" s="35"/>
       <c r="J52" s="16"/>
     </row>
     <row r="53" spans="1:10" ht="30" customHeight="1">
-      <c r="A53" s="30"/>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="30"/>
-      <c r="F53" s="30"/>
-      <c r="G53" s="30"/>
-      <c r="H53" s="30"/>
-      <c r="I53" s="30"/>
+      <c r="A53" s="35"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="35"/>
+      <c r="E53" s="35"/>
+      <c r="F53" s="35"/>
+      <c r="G53" s="35"/>
+      <c r="H53" s="35"/>
+      <c r="I53" s="35"/>
       <c r="J53" s="16"/>
     </row>
     <row r="54" spans="1:10">
@@ -10616,56 +10616,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1"/>
@@ -13460,56 +13460,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1"/>
@@ -13524,18 +13524,18 @@
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="30" t="s">
         <v>186</v>
       </c>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="34"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="1"/>
@@ -16878,56 +16878,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>204</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>205</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1"/>
@@ -17539,81 +17539,81 @@
       <c r="A27" s="2">
         <v>1</v>
       </c>
-      <c r="B27" s="35" t="s">
+      <c r="B27" s="34" t="s">
         <v>246</v>
       </c>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="35"/>
-      <c r="I27" s="35"/>
-      <c r="J27" s="35"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="34"/>
+      <c r="J27" s="34"/>
     </row>
     <row r="28" spans="1:10" ht="30.95" customHeight="1">
       <c r="A28" s="2">
         <v>2</v>
       </c>
-      <c r="B28" s="35" t="s">
+      <c r="B28" s="34" t="s">
         <v>247</v>
       </c>
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="35"/>
-      <c r="I28" s="35"/>
-      <c r="J28" s="35"/>
+      <c r="C28" s="34"/>
+      <c r="D28" s="34"/>
+      <c r="E28" s="34"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="34"/>
+      <c r="J28" s="34"/>
     </row>
     <row r="29" spans="1:10" ht="30.95" customHeight="1">
       <c r="A29" s="2">
         <v>3</v>
       </c>
-      <c r="B29" s="35" t="s">
+      <c r="B29" s="34" t="s">
         <v>248</v>
       </c>
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="34"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
     </row>
     <row r="30" spans="1:10" ht="30.95" customHeight="1">
       <c r="A30" s="2">
         <v>4</v>
       </c>
-      <c r="B30" s="35" t="s">
+      <c r="B30" s="34" t="s">
         <v>249</v>
       </c>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="35"/>
-      <c r="G30" s="35"/>
-      <c r="H30" s="35"/>
-      <c r="I30" s="35"/>
-      <c r="J30" s="35"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="34"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
     </row>
     <row r="31" spans="1:10" ht="30.95" customHeight="1">
       <c r="A31" s="2">
         <v>5</v>
       </c>
-      <c r="B31" s="35" t="s">
+      <c r="B31" s="34" t="s">
         <v>250</v>
       </c>
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="35"/>
-      <c r="F31" s="35"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="35"/>
-      <c r="I31" s="35"/>
-      <c r="J31" s="35"/>
+      <c r="C31" s="34"/>
+      <c r="D31" s="34"/>
+      <c r="E31" s="34"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1"/>
@@ -19672,56 +19672,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="29" t="s">
         <v>252</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="34"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
-      <c r="J2" s="34"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="31" t="s">
         <v>253</v>
       </c>
-      <c r="B3" s="34"/>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="34"/>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
+      <c r="A4" s="30"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" s="1"/>

</xml_diff>